<commit_message>
Cap nhat SELECT thuan va DDL cho CN_266, CN_268, CN_269.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/dashboard/autogen/CN264_270__278_286.xlsx
+++ b/dashboard/autogen/CN264_270__278_286.xlsx
@@ -607,31 +607,20 @@
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>emr_db_tong_hop_luot_kham, emr_db_tong_hop_luot_ra</t>
+          <t>emr_db_tong_hop_luot_vao_ra</t>
         </is>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">SELECT ngay,
-       SUM(so_luot_vao) AS so_luot_vao,
-       SUM(so_luot_ra)  AS so_luot_ra
-FROM (
-    SELECT ngay_vao AS ngay, so_noi_tru AS so_luot_vao, 0 AS so_luot_ra
-    FROM emr_db_tong_hop_luot_kham
-    WHERE ma_csyt = :ma_csyt
-      AND ngay_vao &gt;= :from_date
-      AND ngay_vao &lt; :to_date
-      AND (:thang IS NULL OR thang = :thang)
-    UNION ALL
-    SELECT ngay_ra, 0, so_luot_ra
-    FROM emr_db_tong_hop_luot_ra
-    WHERE ma_csyt = :ma_csyt
-      AND ngay_ra &gt;= :from_date
-      AND ngay_ra &lt; :to_date
-      AND (:thang IS NULL OR thang = :thang)
-) x
-GROUP BY ngay
-ORDER BY ngay
+          <t xml:space="preserve">SELECT ngay_theo_doi AS ngay,
+       so_luot_vao,
+       so_luot_ra
+FROM emr_db_tong_hop_luot_vao_ra
+WHERE ma_csyt = :ma_csyt
+  AND ngay_theo_doi &gt;= :from_date
+  AND ngay_theo_doi &lt; :to_date
+  AND (:thang IS NULL OR thang = :thang)
+ORDER BY ngay_theo_doi
 </t>
         </is>
       </c>
@@ -707,7 +696,7 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>emr_db_tong_hop_luot_kham</t>
+          <t>emr_db_tong_hop_luot_bhyt</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
@@ -715,25 +704,11 @@
           <t xml:space="preserve">SELECT ngay_vao,
        loai,
        luot
-FROM (
-    SELECT ngay_vao,
-           'BHYT' AS loai,
-           so_ho_so_bh AS luot
-    FROM emr_db_tong_hop_luot_kham
-    WHERE ma_csyt = :ma_csyt
-      AND ngay_vao &gt;= :from_date
-      AND ngay_vao &lt; :to_date
-      AND (:thang IS NULL OR thang = :thang)
-    UNION ALL
-    SELECT ngay_vao,
-           'Không BHYT',
-           so_ho_so_khong_bh
-    FROM emr_db_tong_hop_luot_kham
-    WHERE ma_csyt = :ma_csyt
-      AND ngay_vao &gt;= :from_date
-      AND ngay_vao &lt; :to_date
-      AND (:thang IS NULL OR thang = :thang)
-) x
+FROM emr_db_tong_hop_luot_bhyt
+WHERE ma_csyt = :ma_csyt
+  AND ngay_vao &gt;= :from_date
+  AND ngay_vao &lt; :to_date
+  AND (:thang IS NULL OR thang = :thang)
 ORDER BY ngay_vao, loai
 </t>
         </is>
@@ -766,7 +741,7 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>emr_db_tong_hop_luot_kham</t>
+          <t>emr_db_tong_hop_cap_cuu_tu_vong</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
@@ -774,25 +749,11 @@
           <t xml:space="preserve">SELECT ngay_vao,
        loai,
        luot
-FROM (
-    SELECT ngay_vao,
-           'Cấp cứu' AS loai,
-           so_cap_cuu AS luot
-    FROM emr_db_tong_hop_luot_kham
-    WHERE ma_csyt = :ma_csyt
-      AND ngay_vao &gt;= :from_date
-      AND ngay_vao &lt; :to_date
-      AND (:thang IS NULL OR thang = :thang)
-    UNION ALL
-    SELECT ngay_vao,
-           'Tử vong',
-           so_tu_vong
-    FROM emr_db_tong_hop_luot_kham
-    WHERE ma_csyt = :ma_csyt
-      AND ngay_vao &gt;= :from_date
-      AND ngay_vao &lt; :to_date
-      AND (:thang IS NULL OR thang = :thang)
-) x
+FROM emr_db_tong_hop_cap_cuu_tu_vong
+WHERE ma_csyt = :ma_csyt
+  AND ngay_vao &gt;= :from_date
+  AND ngay_vao &lt; :to_date
+  AND (:thang IS NULL OR thang = :thang)
 ORDER BY ngay_vao, loai
 </t>
         </is>

</xml_diff>